<commit_message>
idk what changed here lol
</commit_message>
<xml_diff>
--- a/ASCE 7-16 Seismic Forces-v2.2.xlsx
+++ b/ASCE 7-16 Seismic Forces-v2.2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kpffla-my.sharepoint.com/personal/andy_sazima_kpff_com/Documents/Projects/Beaverton Creek/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="125" documentId="8_{BC827696-9A41-49F6-A0AC-E23791882C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CDC816A-88D0-459A-9289-E7BB4E10D3C8}"/>
+  <xr:revisionPtr revIDLastSave="135" documentId="8_{BC827696-9A41-49F6-A0AC-E23791882C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F851E40-F2B4-4EBD-B5AD-B1507A43D752}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="733" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -102,7 +102,7 @@
     <definedName name="TargetFvE" localSheetId="3">'[1]Site Coefficients (BSE-2N)'!$T$29</definedName>
     <definedName name="TargetFvE">'Site Coefficients'!$U$29</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcCompleted="0"/>
   <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -2994,7 +2994,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="28">
+  <numFmts count="27">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.000\ &quot;g&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
@@ -3022,7 +3022,6 @@
     <numFmt numFmtId="187" formatCode="0.00000"/>
     <numFmt numFmtId="188" formatCode="#,##0.00\ &quot;k&quot;"/>
     <numFmt numFmtId="189" formatCode="#,##0.0000\ &quot;k&quot;"/>
-    <numFmt numFmtId="190" formatCode="#,##0.00000\ &quot;k&quot;"/>
   </numFmts>
   <fonts count="53" x14ac:knownFonts="1">
     <font>
@@ -3720,7 +3719,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="364">
+  <cellXfs count="363">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
@@ -4604,9 +4603,6 @@
     <xf numFmtId="189" fontId="22" fillId="0" borderId="0" xfId="31" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="190" fontId="22" fillId="0" borderId="0" xfId="20" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="187" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5411,10 +5407,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.4</c:v>
+                  <c:v>0.38500000000000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.4</c:v>
+                  <c:v>0.38500000000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6675,10 +6671,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.4</c:v>
+                  <c:v>0.38500000000000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.4</c:v>
+                  <c:v>0.38500000000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8170,9 +8166,9 @@
       <c r="D1" s="207" t="s">
         <v>131</v>
       </c>
-      <c r="E1" s="340"/>
-      <c r="F1" s="341"/>
-      <c r="G1" s="342"/>
+      <c r="E1" s="339"/>
+      <c r="F1" s="340"/>
+      <c r="G1" s="341"/>
       <c r="H1" s="216" t="s">
         <v>132</v>
       </c>
@@ -8208,9 +8204,9 @@
       <c r="D2" s="207" t="s">
         <v>135</v>
       </c>
-      <c r="E2" s="340"/>
-      <c r="F2" s="341"/>
-      <c r="G2" s="342"/>
+      <c r="E2" s="339"/>
+      <c r="F2" s="340"/>
+      <c r="G2" s="341"/>
       <c r="H2" s="216" t="s">
         <v>136</v>
       </c>
@@ -8244,9 +8240,9 @@
       <c r="D3" s="207" t="s">
         <v>138</v>
       </c>
-      <c r="E3" s="340"/>
-      <c r="F3" s="341"/>
-      <c r="G3" s="342"/>
+      <c r="E3" s="339"/>
+      <c r="F3" s="340"/>
+      <c r="G3" s="341"/>
       <c r="H3" s="216" t="s">
         <v>139</v>
       </c>
@@ -8276,11 +8272,11 @@
       <c r="D4" s="207" t="s">
         <v>141</v>
       </c>
-      <c r="E4" s="343" t="s">
+      <c r="E4" s="342" t="s">
         <v>153</v>
       </c>
-      <c r="F4" s="344"/>
-      <c r="G4" s="345"/>
+      <c r="F4" s="343"/>
+      <c r="G4" s="344"/>
       <c r="H4" s="216" t="s">
         <v>136</v>
       </c>
@@ -8332,14 +8328,14 @@
       <c r="H6" s="1"/>
       <c r="J6" s="102"/>
       <c r="K6" s="24"/>
-      <c r="L6" s="339" t="s">
+      <c r="L6" s="338" t="s">
         <v>164</v>
       </c>
-      <c r="M6" s="339"/>
-      <c r="N6" s="339"/>
-      <c r="O6" s="339"/>
-      <c r="P6" s="339"/>
-      <c r="Q6" s="339"/>
+      <c r="M6" s="338"/>
+      <c r="N6" s="338"/>
+      <c r="O6" s="338"/>
+      <c r="P6" s="338"/>
+      <c r="Q6" s="338"/>
       <c r="R6" s="24"/>
       <c r="S6" s="111"/>
       <c r="T6" s="111"/>
@@ -8353,13 +8349,13 @@
       <c r="J7" s="8"/>
       <c r="K7" s="24"/>
       <c r="L7" s="68"/>
-      <c r="M7" s="317" t="s">
+      <c r="M7" s="316" t="s">
         <v>165</v>
       </c>
-      <c r="N7" s="318"/>
-      <c r="O7" s="318"/>
-      <c r="P7" s="318"/>
-      <c r="Q7" s="318"/>
+      <c r="N7" s="317"/>
+      <c r="O7" s="317"/>
+      <c r="P7" s="317"/>
+      <c r="Q7" s="317"/>
       <c r="R7" s="24"/>
       <c r="S7" s="111"/>
       <c r="T7" s="111"/>
@@ -8376,24 +8372,24 @@
       <c r="C8" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="E8" s="336" t="s">
+      <c r="E8" s="335" t="s">
         <v>224</v>
       </c>
-      <c r="F8" s="337"/>
-      <c r="G8" s="337"/>
-      <c r="H8" s="338"/>
+      <c r="F8" s="336"/>
+      <c r="G8" s="336"/>
+      <c r="H8" s="337"/>
       <c r="J8" s="8"/>
       <c r="K8" s="24"/>
       <c r="L8" s="38">
         <v>888</v>
       </c>
-      <c r="M8" s="319" t="s">
+      <c r="M8" s="318" t="s">
         <v>166</v>
       </c>
-      <c r="N8" s="320"/>
-      <c r="O8" s="320"/>
-      <c r="P8" s="320"/>
-      <c r="Q8" s="320"/>
+      <c r="N8" s="319"/>
+      <c r="O8" s="319"/>
+      <c r="P8" s="319"/>
+      <c r="Q8" s="319"/>
       <c r="R8" s="24"/>
       <c r="S8" s="111"/>
       <c r="T8" s="111"/>
@@ -8415,13 +8411,13 @@
       <c r="L9" s="71">
         <v>1.05</v>
       </c>
-      <c r="M9" s="320" t="s">
+      <c r="M9" s="319" t="s">
         <v>167</v>
       </c>
-      <c r="N9" s="320"/>
-      <c r="O9" s="320"/>
-      <c r="P9" s="320"/>
-      <c r="Q9" s="320"/>
+      <c r="N9" s="319"/>
+      <c r="O9" s="319"/>
+      <c r="P9" s="319"/>
+      <c r="Q9" s="319"/>
       <c r="R9" s="24"/>
       <c r="S9" s="111"/>
       <c r="T9" s="111"/>
@@ -8481,12 +8477,12 @@
       <c r="C12" s="41">
         <v>0.88700000000000001</v>
       </c>
-      <c r="E12" s="336" t="s">
+      <c r="E12" s="335" t="s">
         <v>223</v>
       </c>
-      <c r="F12" s="337"/>
-      <c r="G12" s="337"/>
-      <c r="H12" s="338"/>
+      <c r="F12" s="336"/>
+      <c r="G12" s="336"/>
+      <c r="H12" s="337"/>
       <c r="J12" s="8"/>
       <c r="K12" s="24"/>
       <c r="L12" s="24"/>
@@ -8511,12 +8507,12 @@
       <c r="C13" s="41">
         <v>0.41</v>
       </c>
-      <c r="E13" s="336" t="s">
+      <c r="E13" s="335" t="s">
         <v>223</v>
       </c>
-      <c r="F13" s="337"/>
-      <c r="G13" s="337"/>
-      <c r="H13" s="338"/>
+      <c r="F13" s="336"/>
+      <c r="G13" s="336"/>
+      <c r="H13" s="337"/>
       <c r="J13" s="8"/>
       <c r="K13" s="111"/>
       <c r="L13" s="111"/>
@@ -8797,7 +8793,7 @@
       <c r="P22" s="111"/>
       <c r="Q22" s="123">
         <f>C33</f>
-        <v>0.4</v>
+        <v>0.38500000000000001</v>
       </c>
       <c r="R22" s="118">
         <f ca="1">C39</f>
@@ -8833,7 +8829,7 @@
       <c r="P23" s="111"/>
       <c r="Q23" s="125">
         <f>C33</f>
-        <v>0.4</v>
+        <v>0.38500000000000001</v>
       </c>
       <c r="R23" s="126">
         <v>0</v>
@@ -9054,7 +9050,7 @@
         <v>81</v>
       </c>
       <c r="C29" s="74">
-        <v>0.4</v>
+        <v>0.38500000000000001</v>
       </c>
       <c r="E29" s="106" t="s">
         <v>129</v>
@@ -9224,7 +9220,7 @@
       </c>
       <c r="C33" s="76">
         <f>MAX(C29:C31)</f>
-        <v>0.4</v>
+        <v>0.38500000000000001</v>
       </c>
       <c r="E33" s="106" t="s">
         <v>218</v>
@@ -9307,7 +9303,7 @@
       </c>
       <c r="C35" s="103">
         <f ca="1">C21 * (0.4 + 0.6 * C33 / C24)</f>
-        <v>1.3361345998892862</v>
+        <v>1.296187476393438</v>
       </c>
       <c r="E35" s="106" t="s">
         <v>85</v>
@@ -9387,7 +9383,7 @@
       </c>
       <c r="C37" s="103">
         <f ca="1">C22 / C33</f>
-        <v>1.2915000000000001</v>
+        <v>1.341818181818182</v>
       </c>
       <c r="E37" s="109" t="s">
         <v>42</v>
@@ -9427,7 +9423,7 @@
       </c>
       <c r="C38" s="103">
         <f ca="1">C22 * C26 / C33^2</f>
-        <v>51.66</v>
+        <v>55.763872491145229</v>
       </c>
       <c r="E38" s="106" t="s">
         <v>86</v>
@@ -11363,12 +11359,12 @@
       <c r="D1" s="207" t="s">
         <v>131</v>
       </c>
-      <c r="E1" s="346" t="str">
+      <c r="E1" s="345" t="str">
         <f>+IF('Site Ground Motions'!E1="","",'Site Ground Motions'!E1)</f>
         <v/>
       </c>
-      <c r="F1" s="346"/>
-      <c r="G1" s="346"/>
+      <c r="F1" s="345"/>
+      <c r="G1" s="345"/>
       <c r="H1" s="216" t="s">
         <v>132</v>
       </c>
@@ -11408,12 +11404,12 @@
       <c r="D2" s="207" t="s">
         <v>135</v>
       </c>
-      <c r="E2" s="346" t="str">
+      <c r="E2" s="345" t="str">
         <f>+IF('Site Ground Motions'!E2="","",'Site Ground Motions'!E2)</f>
         <v/>
       </c>
-      <c r="F2" s="346"/>
-      <c r="G2" s="346"/>
+      <c r="F2" s="345"/>
+      <c r="G2" s="345"/>
       <c r="H2" s="216" t="s">
         <v>136</v>
       </c>
@@ -11453,12 +11449,12 @@
       <c r="D3" s="207" t="s">
         <v>138</v>
       </c>
-      <c r="E3" s="346" t="str">
+      <c r="E3" s="345" t="str">
         <f>+IF('Site Ground Motions'!E3="","",'Site Ground Motions'!E3)</f>
         <v/>
       </c>
-      <c r="F3" s="346"/>
-      <c r="G3" s="346"/>
+      <c r="F3" s="345"/>
+      <c r="G3" s="345"/>
       <c r="H3" s="216" t="s">
         <v>139</v>
       </c>
@@ -11491,11 +11487,11 @@
       <c r="D4" s="207" t="s">
         <v>141</v>
       </c>
-      <c r="E4" s="346" t="s">
+      <c r="E4" s="345" t="s">
         <v>176</v>
       </c>
-      <c r="F4" s="346"/>
-      <c r="G4" s="346"/>
+      <c r="F4" s="345"/>
+      <c r="G4" s="345"/>
       <c r="H4" s="216" t="s">
         <v>136</v>
       </c>
@@ -11508,16 +11504,16 @@
         <v/>
       </c>
       <c r="K4" s="24"/>
-      <c r="L4" s="339" t="s">
+      <c r="L4" s="338" t="s">
         <v>164</v>
       </c>
-      <c r="M4" s="339"/>
-      <c r="N4" s="339"/>
-      <c r="O4" s="339"/>
-      <c r="P4" s="339"/>
-      <c r="Q4" s="339"/>
-      <c r="R4" s="339"/>
-      <c r="S4" s="339"/>
+      <c r="M4" s="338"/>
+      <c r="N4" s="338"/>
+      <c r="O4" s="338"/>
+      <c r="P4" s="338"/>
+      <c r="Q4" s="338"/>
+      <c r="R4" s="338"/>
+      <c r="S4" s="338"/>
       <c r="T4" s="111"/>
       <c r="U4" s="111"/>
       <c r="V4" s="111"/>
@@ -11537,15 +11533,15 @@
       <c r="J5" s="44"/>
       <c r="K5" s="24"/>
       <c r="L5" s="68"/>
-      <c r="M5" s="317" t="s">
+      <c r="M5" s="316" t="s">
         <v>165</v>
       </c>
-      <c r="N5" s="318"/>
-      <c r="O5" s="318"/>
-      <c r="P5" s="318"/>
-      <c r="Q5" s="318"/>
-      <c r="R5" s="318"/>
-      <c r="S5" s="318"/>
+      <c r="N5" s="317"/>
+      <c r="O5" s="317"/>
+      <c r="P5" s="317"/>
+      <c r="Q5" s="317"/>
+      <c r="R5" s="317"/>
+      <c r="S5" s="317"/>
       <c r="T5" s="111"/>
       <c r="U5" s="111"/>
       <c r="V5" s="111"/>
@@ -11567,15 +11563,15 @@
       <c r="L6" s="38">
         <v>888</v>
       </c>
-      <c r="M6" s="319" t="s">
+      <c r="M6" s="318" t="s">
         <v>166</v>
       </c>
-      <c r="N6" s="320"/>
-      <c r="O6" s="320"/>
-      <c r="P6" s="320"/>
-      <c r="Q6" s="320"/>
-      <c r="R6" s="320"/>
-      <c r="S6" s="320"/>
+      <c r="N6" s="319"/>
+      <c r="O6" s="319"/>
+      <c r="P6" s="319"/>
+      <c r="Q6" s="319"/>
+      <c r="R6" s="319"/>
+      <c r="S6" s="319"/>
       <c r="T6" s="111"/>
       <c r="U6" s="111"/>
       <c r="V6" s="111"/>
@@ -11589,15 +11585,15 @@
       <c r="L7" s="71">
         <v>1.05</v>
       </c>
-      <c r="M7" s="320" t="s">
+      <c r="M7" s="319" t="s">
         <v>167</v>
       </c>
-      <c r="N7" s="320"/>
-      <c r="O7" s="320"/>
-      <c r="P7" s="320"/>
-      <c r="Q7" s="320"/>
-      <c r="R7" s="320"/>
-      <c r="S7" s="320"/>
+      <c r="N7" s="319"/>
+      <c r="O7" s="319"/>
+      <c r="P7" s="319"/>
+      <c r="Q7" s="319"/>
+      <c r="R7" s="319"/>
+      <c r="S7" s="319"/>
       <c r="T7" s="111"/>
       <c r="U7" s="111"/>
       <c r="V7" s="111"/>
@@ -11666,13 +11662,13 @@
     <row r="10" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="48"/>
       <c r="B10" s="20"/>
-      <c r="C10" s="356" t="s">
+      <c r="C10" s="355" t="s">
         <v>78</v>
       </c>
-      <c r="D10" s="357"/>
-      <c r="E10" s="357"/>
-      <c r="F10" s="357"/>
-      <c r="G10" s="358"/>
+      <c r="D10" s="356"/>
+      <c r="E10" s="356"/>
+      <c r="F10" s="356"/>
+      <c r="G10" s="357"/>
       <c r="J10" s="47"/>
       <c r="K10" s="136"/>
       <c r="L10" s="137">
@@ -11712,13 +11708,13 @@
     <row r="11" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="48"/>
       <c r="B11" s="19"/>
-      <c r="C11" s="353" t="s">
+      <c r="C11" s="352" t="s">
         <v>79</v>
       </c>
-      <c r="D11" s="354"/>
-      <c r="E11" s="354"/>
-      <c r="F11" s="354"/>
-      <c r="G11" s="355"/>
+      <c r="D11" s="353"/>
+      <c r="E11" s="353"/>
+      <c r="F11" s="353"/>
+      <c r="G11" s="354"/>
       <c r="J11" s="47"/>
       <c r="K11" s="302" t="s">
         <v>221</v>
@@ -12065,11 +12061,11 @@
       <c r="E17" s="17">
         <v>1.3</v>
       </c>
-      <c r="F17" s="359" t="s">
+      <c r="F17" s="358" t="s">
         <v>119</v>
       </c>
-      <c r="G17" s="360"/>
-      <c r="H17" s="361"/>
+      <c r="G17" s="359"/>
+      <c r="H17" s="360"/>
       <c r="J17" s="47"/>
       <c r="K17" s="138"/>
       <c r="L17" s="139" t="s">
@@ -12116,14 +12112,14 @@
       <c r="B18" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="350" t="s">
+      <c r="C18" s="349" t="s">
         <v>119</v>
       </c>
-      <c r="D18" s="351"/>
-      <c r="E18" s="351"/>
-      <c r="F18" s="351"/>
-      <c r="G18" s="351"/>
-      <c r="H18" s="352"/>
+      <c r="D18" s="350"/>
+      <c r="E18" s="350"/>
+      <c r="F18" s="350"/>
+      <c r="G18" s="350"/>
+      <c r="H18" s="351"/>
       <c r="J18" s="47"/>
       <c r="K18" s="138"/>
       <c r="L18" s="139" t="s">
@@ -12285,13 +12281,13 @@
     <row r="23" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="48"/>
       <c r="B23" s="20"/>
-      <c r="C23" s="356" t="s">
+      <c r="C23" s="355" t="s">
         <v>78</v>
       </c>
-      <c r="D23" s="357"/>
-      <c r="E23" s="357"/>
-      <c r="F23" s="357"/>
-      <c r="G23" s="358"/>
+      <c r="D23" s="356"/>
+      <c r="E23" s="356"/>
+      <c r="F23" s="356"/>
+      <c r="G23" s="357"/>
       <c r="J23" s="47"/>
       <c r="K23" s="136"/>
       <c r="L23" s="137">
@@ -12331,13 +12327,13 @@
     <row r="24" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="48"/>
       <c r="B24" s="19"/>
-      <c r="C24" s="353" t="s">
+      <c r="C24" s="352" t="s">
         <v>80</v>
       </c>
-      <c r="D24" s="354"/>
-      <c r="E24" s="354"/>
-      <c r="F24" s="354"/>
-      <c r="G24" s="355"/>
+      <c r="D24" s="353"/>
+      <c r="E24" s="353"/>
+      <c r="F24" s="353"/>
+      <c r="G24" s="354"/>
       <c r="J24" s="47"/>
       <c r="K24" s="136"/>
       <c r="L24" s="137">
@@ -12672,13 +12668,13 @@
       <c r="C30" s="17">
         <v>4.2</v>
       </c>
-      <c r="D30" s="347" t="s">
+      <c r="D30" s="346" t="s">
         <v>119</v>
       </c>
-      <c r="E30" s="348"/>
-      <c r="F30" s="348"/>
-      <c r="G30" s="348"/>
-      <c r="H30" s="349"/>
+      <c r="E30" s="347"/>
+      <c r="F30" s="347"/>
+      <c r="G30" s="347"/>
+      <c r="H30" s="348"/>
       <c r="J30" s="47"/>
       <c r="K30" s="136"/>
       <c r="L30" s="139" t="s">
@@ -12725,14 +12721,14 @@
       <c r="B31" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="C31" s="350" t="s">
+      <c r="C31" s="349" t="s">
         <v>119</v>
       </c>
-      <c r="D31" s="351"/>
-      <c r="E31" s="351"/>
-      <c r="F31" s="351"/>
-      <c r="G31" s="351"/>
-      <c r="H31" s="352"/>
+      <c r="D31" s="350"/>
+      <c r="E31" s="350"/>
+      <c r="F31" s="350"/>
+      <c r="G31" s="350"/>
+      <c r="H31" s="351"/>
       <c r="J31" s="47"/>
       <c r="K31" s="136"/>
       <c r="L31" s="139" t="s">
@@ -20175,15 +20171,15 @@
       <c r="D1" s="197" t="s">
         <v>131</v>
       </c>
-      <c r="E1" s="362" t="str">
+      <c r="E1" s="361" t="str">
         <f>+IF('Site Ground Motions'!E1="","",'Site Ground Motions'!E1)</f>
         <v/>
       </c>
-      <c r="F1" s="362"/>
-      <c r="G1" s="362"/>
-      <c r="H1" s="362"/>
-      <c r="I1" s="362"/>
-      <c r="J1" s="362"/>
+      <c r="F1" s="361"/>
+      <c r="G1" s="361"/>
+      <c r="H1" s="361"/>
+      <c r="I1" s="361"/>
+      <c r="J1" s="361"/>
       <c r="K1" s="219" t="s">
         <v>132</v>
       </c>
@@ -20222,15 +20218,15 @@
       <c r="D2" s="197" t="s">
         <v>135</v>
       </c>
-      <c r="E2" s="362" t="str">
+      <c r="E2" s="361" t="str">
         <f>+IF('Site Ground Motions'!E2="","",'Site Ground Motions'!E2)</f>
         <v/>
       </c>
-      <c r="F2" s="362"/>
-      <c r="G2" s="362"/>
-      <c r="H2" s="362"/>
-      <c r="I2" s="362"/>
-      <c r="J2" s="362"/>
+      <c r="F2" s="361"/>
+      <c r="G2" s="361"/>
+      <c r="H2" s="361"/>
+      <c r="I2" s="361"/>
+      <c r="J2" s="361"/>
       <c r="K2" s="219" t="s">
         <v>136</v>
       </c>
@@ -20269,15 +20265,15 @@
       <c r="D3" s="197" t="s">
         <v>138</v>
       </c>
-      <c r="E3" s="362" t="str">
+      <c r="E3" s="361" t="str">
         <f>+IF('Site Ground Motions'!E3="","",'Site Ground Motions'!E3)</f>
         <v/>
       </c>
-      <c r="F3" s="362"/>
-      <c r="G3" s="362"/>
-      <c r="H3" s="362"/>
-      <c r="I3" s="362"/>
-      <c r="J3" s="362"/>
+      <c r="F3" s="361"/>
+      <c r="G3" s="361"/>
+      <c r="H3" s="361"/>
+      <c r="I3" s="361"/>
+      <c r="J3" s="361"/>
       <c r="K3" s="219" t="s">
         <v>139</v>
       </c>
@@ -20309,14 +20305,14 @@
       <c r="D4" s="197" t="s">
         <v>141</v>
       </c>
-      <c r="E4" s="362" t="s">
+      <c r="E4" s="361" t="s">
         <v>175</v>
       </c>
-      <c r="F4" s="362"/>
-      <c r="G4" s="362"/>
-      <c r="H4" s="362"/>
-      <c r="I4" s="362"/>
-      <c r="J4" s="362"/>
+      <c r="F4" s="361"/>
+      <c r="G4" s="361"/>
+      <c r="H4" s="361"/>
+      <c r="I4" s="361"/>
+      <c r="J4" s="361"/>
       <c r="K4" s="219" t="s">
         <v>136</v>
       </c>
@@ -20329,16 +20325,16 @@
         <v/>
       </c>
       <c r="N4" s="24"/>
-      <c r="O4" s="339" t="s">
+      <c r="O4" s="338" t="s">
         <v>164</v>
       </c>
-      <c r="P4" s="339"/>
-      <c r="Q4" s="339"/>
-      <c r="R4" s="339"/>
-      <c r="S4" s="339"/>
-      <c r="T4" s="339"/>
-      <c r="U4" s="339"/>
-      <c r="V4" s="339"/>
+      <c r="P4" s="338"/>
+      <c r="Q4" s="338"/>
+      <c r="R4" s="338"/>
+      <c r="S4" s="338"/>
+      <c r="T4" s="338"/>
+      <c r="U4" s="338"/>
+      <c r="V4" s="338"/>
       <c r="W4" s="111"/>
       <c r="X4" s="111"/>
       <c r="Y4" s="111"/>
@@ -20349,15 +20345,15 @@
       <c r="M5" s="8"/>
       <c r="N5" s="24"/>
       <c r="O5" s="68"/>
-      <c r="P5" s="317" t="s">
+      <c r="P5" s="316" t="s">
         <v>165</v>
       </c>
-      <c r="Q5" s="318"/>
-      <c r="R5" s="318"/>
-      <c r="S5" s="318"/>
-      <c r="T5" s="318"/>
-      <c r="U5" s="318"/>
-      <c r="V5" s="318"/>
+      <c r="Q5" s="317"/>
+      <c r="R5" s="317"/>
+      <c r="S5" s="317"/>
+      <c r="T5" s="317"/>
+      <c r="U5" s="317"/>
+      <c r="V5" s="317"/>
       <c r="W5" s="111"/>
       <c r="X5" s="111"/>
       <c r="Y5" s="111"/>
@@ -20381,15 +20377,15 @@
       <c r="O6" s="38">
         <v>888</v>
       </c>
-      <c r="P6" s="319" t="s">
+      <c r="P6" s="318" t="s">
         <v>166</v>
       </c>
-      <c r="Q6" s="320"/>
-      <c r="R6" s="320"/>
-      <c r="S6" s="320"/>
-      <c r="T6" s="320"/>
-      <c r="U6" s="320"/>
-      <c r="V6" s="320"/>
+      <c r="Q6" s="319"/>
+      <c r="R6" s="319"/>
+      <c r="S6" s="319"/>
+      <c r="T6" s="319"/>
+      <c r="U6" s="319"/>
+      <c r="V6" s="319"/>
       <c r="W6" s="111"/>
       <c r="X6" s="111"/>
       <c r="Y6" s="111"/>
@@ -20402,15 +20398,15 @@
       <c r="O7" s="71">
         <v>1.05</v>
       </c>
-      <c r="P7" s="320" t="s">
+      <c r="P7" s="319" t="s">
         <v>167</v>
       </c>
-      <c r="Q7" s="320"/>
-      <c r="R7" s="320"/>
-      <c r="S7" s="320"/>
-      <c r="T7" s="320"/>
-      <c r="U7" s="320"/>
-      <c r="V7" s="320"/>
+      <c r="Q7" s="319"/>
+      <c r="R7" s="319"/>
+      <c r="S7" s="319"/>
+      <c r="T7" s="319"/>
+      <c r="U7" s="319"/>
+      <c r="V7" s="319"/>
       <c r="W7" s="111"/>
       <c r="X7" s="111"/>
       <c r="Y7" s="111"/>
@@ -20531,7 +20527,7 @@
       <c r="U12" s="111"/>
       <c r="V12" s="123">
         <f>'Site Ground Motions'!Q22</f>
-        <v>0.4</v>
+        <v>0.38500000000000001</v>
       </c>
       <c r="W12" s="150">
         <f ca="1">'Site Ground Motions'!R22</f>
@@ -20565,7 +20561,7 @@
       </c>
       <c r="I13" s="95">
         <f>'Site Ground Motions'!C33</f>
-        <v>0.4</v>
+        <v>0.38500000000000001</v>
       </c>
       <c r="K13" s="11"/>
       <c r="L13" s="90"/>
@@ -20585,7 +20581,7 @@
       <c r="U13" s="111"/>
       <c r="V13" s="125">
         <f>'Site Ground Motions'!Q23</f>
-        <v>0.4</v>
+        <v>0.38500000000000001</v>
       </c>
       <c r="W13" s="153">
         <f>'Site Ground Motions'!R23</f>
@@ -20951,7 +20947,7 @@
       </c>
       <c r="D25" s="99">
         <f ca="1">C14 / I13 / D22</f>
-        <v>0.1986923076923077</v>
+        <v>0.20643356643356647</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>91</v>
@@ -20993,7 +20989,7 @@
       </c>
       <c r="D26" s="99">
         <f ca="1">1.5*C14 / I13 / D22</f>
-        <v>0.29803846153846159</v>
+        <v>0.30965034965034971</v>
       </c>
       <c r="F26" s="10" t="s">
         <v>120</v>
@@ -21035,7 +21031,7 @@
       </c>
       <c r="D27" s="99">
         <f ca="1">C14 * F15 / I13^2 / D22</f>
-        <v>7.9476923076923072</v>
+        <v>8.5790573063300357</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>92</v>
@@ -21077,7 +21073,7 @@
       </c>
       <c r="D28" s="99">
         <f ca="1">1.5*C14 * F15 / I13^2 / D22</f>
-        <v>11.921538461538461</v>
+        <v>12.868585959495052</v>
       </c>
       <c r="F28" s="10" t="s">
         <v>121</v>
@@ -21234,7 +21230,7 @@
       <c r="C32" s="91" t="s">
         <v>19</v>
       </c>
-      <c r="D32" s="310">
+      <c r="D32" s="309">
         <f ca="1">O17</f>
         <v>0.10418383589743591</v>
       </c>
@@ -23182,14 +23178,14 @@
       <c r="E1" s="197" t="s">
         <v>131</v>
       </c>
-      <c r="F1" s="331" t="str">
+      <c r="F1" s="330" t="str">
         <f>+IF('Site Ground Motions'!E1="","",'Site Ground Motions'!E1)</f>
         <v/>
       </c>
-      <c r="G1" s="332"/>
-      <c r="H1" s="332"/>
-      <c r="I1" s="332"/>
-      <c r="J1" s="333"/>
+      <c r="G1" s="331"/>
+      <c r="H1" s="331"/>
+      <c r="I1" s="331"/>
+      <c r="J1" s="332"/>
       <c r="K1" s="219" t="s">
         <v>132</v>
       </c>
@@ -23229,14 +23225,14 @@
       <c r="E2" s="197" t="s">
         <v>135</v>
       </c>
-      <c r="F2" s="331" t="str">
+      <c r="F2" s="330" t="str">
         <f>+IF('Site Ground Motions'!E2="","",'Site Ground Motions'!E2)</f>
         <v/>
       </c>
-      <c r="G2" s="332"/>
-      <c r="H2" s="332"/>
-      <c r="I2" s="332"/>
-      <c r="J2" s="333"/>
+      <c r="G2" s="331"/>
+      <c r="H2" s="331"/>
+      <c r="I2" s="331"/>
+      <c r="J2" s="332"/>
       <c r="K2" s="219" t="s">
         <v>136</v>
       </c>
@@ -23276,14 +23272,14 @@
       <c r="E3" s="197" t="s">
         <v>138</v>
       </c>
-      <c r="F3" s="331" t="str">
+      <c r="F3" s="330" t="str">
         <f>+IF('Site Ground Motions'!E3="","",'Site Ground Motions'!E3)</f>
         <v/>
       </c>
-      <c r="G3" s="332"/>
-      <c r="H3" s="332"/>
-      <c r="I3" s="332"/>
-      <c r="J3" s="333"/>
+      <c r="G3" s="331"/>
+      <c r="H3" s="331"/>
+      <c r="I3" s="331"/>
+      <c r="J3" s="332"/>
       <c r="K3" s="219" t="s">
         <v>139</v>
       </c>
@@ -23316,13 +23312,13 @@
       <c r="E4" s="197" t="s">
         <v>141</v>
       </c>
-      <c r="F4" s="331" t="s">
+      <c r="F4" s="330" t="s">
         <v>154</v>
       </c>
-      <c r="G4" s="332"/>
-      <c r="H4" s="332"/>
-      <c r="I4" s="332"/>
-      <c r="J4" s="333"/>
+      <c r="G4" s="331"/>
+      <c r="H4" s="331"/>
+      <c r="I4" s="331"/>
+      <c r="J4" s="332"/>
       <c r="K4" s="219" t="s">
         <v>136</v>
       </c>
@@ -23350,17 +23346,17 @@
     </row>
     <row r="5" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="28"/>
-      <c r="B5" s="334" t="s">
+      <c r="B5" s="333" t="s">
         <v>152</v>
       </c>
-      <c r="C5" s="334"/>
-      <c r="D5" s="334"/>
-      <c r="E5" s="334"/>
-      <c r="F5" s="334"/>
-      <c r="G5" s="334"/>
-      <c r="H5" s="334"/>
-      <c r="I5" s="334"/>
-      <c r="J5" s="334"/>
+      <c r="C5" s="333"/>
+      <c r="D5" s="333"/>
+      <c r="E5" s="333"/>
+      <c r="F5" s="333"/>
+      <c r="G5" s="333"/>
+      <c r="H5" s="333"/>
+      <c r="I5" s="333"/>
+      <c r="J5" s="333"/>
       <c r="K5" s="233"/>
       <c r="L5" s="233"/>
       <c r="M5" s="33"/>
@@ -23380,28 +23376,28 @@
     </row>
     <row r="6" spans="1:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="35"/>
-      <c r="B6" s="335"/>
-      <c r="C6" s="335"/>
-      <c r="D6" s="335"/>
-      <c r="E6" s="335"/>
-      <c r="F6" s="335"/>
-      <c r="G6" s="335"/>
-      <c r="H6" s="335"/>
-      <c r="I6" s="335"/>
-      <c r="J6" s="335"/>
+      <c r="B6" s="334"/>
+      <c r="C6" s="334"/>
+      <c r="D6" s="334"/>
+      <c r="E6" s="334"/>
+      <c r="F6" s="334"/>
+      <c r="G6" s="334"/>
+      <c r="H6" s="334"/>
+      <c r="I6" s="334"/>
+      <c r="J6" s="334"/>
       <c r="K6" s="233"/>
       <c r="L6" s="233"/>
       <c r="M6" s="33"/>
       <c r="N6" s="24"/>
-      <c r="O6" s="316" t="s">
+      <c r="O6" s="315" t="s">
         <v>164</v>
       </c>
-      <c r="P6" s="316"/>
-      <c r="Q6" s="316"/>
-      <c r="R6" s="316"/>
-      <c r="S6" s="316"/>
-      <c r="T6" s="316"/>
-      <c r="U6" s="316"/>
+      <c r="P6" s="315"/>
+      <c r="Q6" s="315"/>
+      <c r="R6" s="315"/>
+      <c r="S6" s="315"/>
+      <c r="T6" s="315"/>
+      <c r="U6" s="315"/>
       <c r="V6" s="24"/>
       <c r="W6" s="24"/>
       <c r="X6" s="24"/>
@@ -23424,14 +23420,14 @@
       <c r="M7" s="33"/>
       <c r="N7" s="24"/>
       <c r="O7" s="68"/>
-      <c r="P7" s="317" t="s">
+      <c r="P7" s="316" t="s">
         <v>165</v>
       </c>
-      <c r="Q7" s="318"/>
-      <c r="R7" s="318"/>
-      <c r="S7" s="318"/>
-      <c r="T7" s="318"/>
-      <c r="U7" s="318"/>
+      <c r="Q7" s="317"/>
+      <c r="R7" s="317"/>
+      <c r="S7" s="317"/>
+      <c r="T7" s="317"/>
+      <c r="U7" s="317"/>
       <c r="V7" s="24"/>
       <c r="W7" s="24"/>
       <c r="X7" s="24"/>
@@ -23447,7 +23443,7 @@
       </c>
       <c r="E8" s="235">
         <f>+'Site Ground Motions'!C33</f>
-        <v>0.4</v>
+        <v>0.38500000000000001</v>
       </c>
       <c r="F8" s="232"/>
       <c r="G8" s="234" t="s">
@@ -23468,14 +23464,14 @@
       <c r="O8" s="38">
         <v>888</v>
       </c>
-      <c r="P8" s="319" t="s">
+      <c r="P8" s="318" t="s">
         <v>166</v>
       </c>
-      <c r="Q8" s="320"/>
-      <c r="R8" s="320"/>
-      <c r="S8" s="320"/>
-      <c r="T8" s="320"/>
-      <c r="U8" s="320"/>
+      <c r="Q8" s="319"/>
+      <c r="R8" s="319"/>
+      <c r="S8" s="319"/>
+      <c r="T8" s="319"/>
+      <c r="U8" s="319"/>
       <c r="V8" s="24"/>
       <c r="W8" s="24"/>
       <c r="X8" s="24"/>
@@ -23489,9 +23485,9 @@
       <c r="D9" s="234" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="309">
+      <c r="E9" s="181">
         <f>F18</f>
-        <v>2100.8365000000003</v>
+        <v>2057.489</v>
       </c>
       <c r="F9" s="232"/>
       <c r="G9" s="237"/>
@@ -23505,14 +23501,14 @@
       <c r="O9" s="71">
         <v>1.05</v>
       </c>
-      <c r="P9" s="320" t="s">
+      <c r="P9" s="319" t="s">
         <v>167</v>
       </c>
-      <c r="Q9" s="320"/>
-      <c r="R9" s="320"/>
-      <c r="S9" s="320"/>
-      <c r="T9" s="320"/>
-      <c r="U9" s="320"/>
+      <c r="Q9" s="319"/>
+      <c r="R9" s="319"/>
+      <c r="S9" s="319"/>
+      <c r="T9" s="319"/>
+      <c r="U9" s="319"/>
       <c r="V9" s="24"/>
       <c r="W9" s="24"/>
       <c r="X9" s="24"/>
@@ -23603,7 +23599,7 @@
       </c>
       <c r="I12" s="178">
         <f ca="1">I11 * E9</f>
-        <v>218.87320516334364</v>
+        <v>214.35709633677951</v>
       </c>
       <c r="J12" s="240"/>
       <c r="K12" s="232"/>
@@ -23680,18 +23676,18 @@
     <row r="15" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="35"/>
       <c r="B15" s="232"/>
-      <c r="C15" s="321" t="s">
+      <c r="C15" s="320" t="s">
         <v>154</v>
       </c>
-      <c r="D15" s="321"/>
-      <c r="E15" s="321"/>
-      <c r="F15" s="321"/>
-      <c r="G15" s="321"/>
-      <c r="H15" s="321"/>
-      <c r="I15" s="321"/>
-      <c r="J15" s="321"/>
-      <c r="K15" s="321"/>
-      <c r="L15" s="321"/>
+      <c r="D15" s="320"/>
+      <c r="E15" s="320"/>
+      <c r="F15" s="320"/>
+      <c r="G15" s="320"/>
+      <c r="H15" s="320"/>
+      <c r="I15" s="320"/>
+      <c r="J15" s="320"/>
+      <c r="K15" s="320"/>
+      <c r="L15" s="320"/>
       <c r="M15" s="77"/>
       <c r="N15" s="24"/>
       <c r="Q15" s="24"/>
@@ -23756,8 +23752,8 @@
         <v>190</v>
       </c>
       <c r="J17" s="78"/>
-      <c r="K17" s="322"/>
-      <c r="L17" s="322"/>
+      <c r="K17" s="321"/>
+      <c r="L17" s="321"/>
       <c r="M17" s="77"/>
       <c r="N17" s="24"/>
       <c r="O17" s="24"/>
@@ -23784,11 +23780,11 @@
       <c r="E18" s="232"/>
       <c r="F18" s="181">
         <f>SUM(F24:F36)</f>
-        <v>2100.8365000000003</v>
+        <v>2057.489</v>
       </c>
       <c r="G18" s="181">
         <f>SUM(G24:G36)</f>
-        <v>54984.912500000006</v>
+        <v>53848.225000000006</v>
       </c>
       <c r="H18" s="257">
         <f>SUM(H24:H36)</f>
@@ -23796,7 +23792,7 @@
       </c>
       <c r="I18" s="178">
         <f ca="1">SUM(I24:I36)</f>
-        <v>218.87320516334364</v>
+        <v>214.35709633677948</v>
       </c>
       <c r="J18" s="232"/>
       <c r="K18" s="232"/>
@@ -23854,20 +23850,20 @@
       </c>
       <c r="F20" s="229">
         <f ca="1">MAX(K25:K32) / I12</f>
-        <v>31.031679808529297</v>
-      </c>
-      <c r="G20" s="311" t="s">
+        <v>31.030566262861957</v>
+      </c>
+      <c r="G20" s="310" t="s">
         <v>148</v>
       </c>
-      <c r="H20" s="311"/>
+      <c r="H20" s="310"/>
       <c r="I20" s="258">
         <f ca="1">F20 / D18</f>
-        <v>0.7301571719653952</v>
-      </c>
-      <c r="J20" s="311" t="s">
+        <v>0.73013097089086954</v>
+      </c>
+      <c r="J20" s="310" t="s">
         <v>149</v>
       </c>
-      <c r="K20" s="311"/>
+      <c r="K20" s="310"/>
       <c r="L20" s="232"/>
       <c r="M20" s="77"/>
       <c r="N20" s="24"/>
@@ -23973,10 +23969,10 @@
       <c r="J23" s="78" t="s">
         <v>172</v>
       </c>
-      <c r="K23" s="322" t="s">
+      <c r="K23" s="321" t="s">
         <v>32</v>
       </c>
-      <c r="L23" s="322"/>
+      <c r="L23" s="321"/>
       <c r="M23" s="77"/>
       <c r="N23" s="24"/>
       <c r="O23" s="24"/>
@@ -24006,31 +24002,31 @@
         <v>42.5</v>
       </c>
       <c r="F24" s="193">
-        <v>430.46499999999997</v>
+        <v>421.49</v>
       </c>
       <c r="G24" s="181">
         <f>F24 * (E24-E$12)^$H$8</f>
-        <v>18294.762500000001</v>
+        <v>17913.325000000001</v>
       </c>
       <c r="H24" s="230">
         <f>G24 / $G$18</f>
-        <v>0.3327233175100533</v>
+        <v>0.33266324006037334</v>
       </c>
       <c r="I24" s="306">
         <f ca="1">H24 * $I$12</f>
-        <v>72.824218936006218</v>
+        <v>71.308726197326649</v>
       </c>
       <c r="J24" s="83" t="s">
         <v>151</v>
       </c>
-      <c r="K24" s="326" t="s">
+      <c r="K24" s="325" t="s">
         <v>151</v>
       </c>
-      <c r="L24" s="326"/>
+      <c r="L24" s="325"/>
       <c r="M24" s="77"/>
       <c r="N24" s="24"/>
       <c r="O24" s="225"/>
-      <c r="P24" s="323" t="s">
+      <c r="P24" s="322" t="s">
         <v>212</v>
       </c>
       <c r="Q24" s="24"/>
@@ -24059,35 +24055,35 @@
         <v>32.5</v>
       </c>
       <c r="F25" s="84">
-        <v>554.33450000000005</v>
+        <v>542.91700000000003</v>
       </c>
       <c r="G25" s="181">
         <f t="shared" ref="G25:G27" si="1">IF(C25="","",IF(C25="Ground","—",F25 * (E25-E$12)^$H$8))</f>
-        <v>18015.87125</v>
+        <v>17644.802500000002</v>
       </c>
       <c r="H25" s="230">
         <f>IF(C25="","",IF(C25="Ground","—",G25 / $G$18))</f>
-        <v>0.32765117612945183</v>
+        <v>0.32767658543991002</v>
       </c>
       <c r="I25" s="306">
         <f ca="1">IF(C25="","",IF(C25="Ground","—",H25 * $I$12))</f>
-        <v>71.714063094992355</v>
+        <v>70.239801392449749</v>
       </c>
       <c r="J25" s="307">
         <f ca="1">IF(C25="","",IF(C25="Ground","—",I24))</f>
-        <v>72.824218936006218</v>
-      </c>
-      <c r="K25" s="314">
+        <v>71.308726197326649</v>
+      </c>
+      <c r="K25" s="313">
         <f ca="1">IF(C25="","",J25 * D25)</f>
-        <v>728.24218936006218</v>
-      </c>
-      <c r="L25" s="314"/>
+        <v>713.08726197326655</v>
+      </c>
+      <c r="L25" s="313"/>
       <c r="M25" s="194"/>
       <c r="N25" s="24"/>
       <c r="O25" s="226" t="s">
         <v>186</v>
       </c>
-      <c r="P25" s="324"/>
+      <c r="P25" s="323"/>
       <c r="Q25" s="24"/>
       <c r="R25" s="24"/>
       <c r="S25" s="24"/>
@@ -24114,35 +24110,35 @@
         <v>22</v>
       </c>
       <c r="F26" s="84">
-        <v>556.17650000000003</v>
+        <v>544.72900000000004</v>
       </c>
       <c r="G26" s="181">
         <f t="shared" si="1"/>
-        <v>12235.883000000002</v>
+        <v>11984.038</v>
       </c>
       <c r="H26" s="230">
         <f>IF(C26="","",IF(C26="Ground","—",G26 / $G$18))</f>
-        <v>0.22253164447610971</v>
+        <v>0.2225521454049785</v>
       </c>
       <c r="I26" s="306">
         <f t="shared" ref="I26:I27" ca="1" si="3">IF(C26="","",IF(C26="Ground","—",H26 * $I$12))</f>
-        <v>48.706214276755809</v>
+        <v>47.705631672531936</v>
       </c>
       <c r="J26" s="307">
         <f t="shared" ref="J26:J27" ca="1" si="4">IF(C26="","",I25+J25)</f>
-        <v>144.53828203099857</v>
-      </c>
-      <c r="K26" s="314">
+        <v>141.5485275897764</v>
+      </c>
+      <c r="K26" s="313">
         <f t="shared" ref="K26:K27" ca="1" si="5">IF(C26="","",J26 * D26+K25)</f>
-        <v>2245.8941506855472</v>
-      </c>
-      <c r="L26" s="314"/>
+        <v>2199.346801665919</v>
+      </c>
+      <c r="L26" s="313"/>
       <c r="M26" s="194"/>
       <c r="N26" s="24"/>
       <c r="O26" s="226">
         <v>1</v>
       </c>
-      <c r="P26" s="324"/>
+      <c r="P26" s="323"/>
       <c r="Q26" s="24"/>
       <c r="R26" s="24"/>
       <c r="S26" s="24"/>
@@ -24169,35 +24165,35 @@
         <v>11.5</v>
       </c>
       <c r="F27" s="84">
-        <v>559.8605</v>
+        <v>548.35299999999995</v>
       </c>
       <c r="G27" s="181">
         <f t="shared" si="1"/>
-        <v>6438.3957499999997</v>
+        <v>6306.0594999999994</v>
       </c>
       <c r="H27" s="230">
         <f>IF(C27="","",IF(C27="Ground","—",G27 / $G$18))</f>
-        <v>0.11709386188438509</v>
+        <v>0.11710802909473801</v>
       </c>
       <c r="I27" s="306">
         <f t="shared" ca="1" si="3"/>
-        <v>25.628708855589242</v>
+        <v>25.102937074471132</v>
       </c>
       <c r="J27" s="307">
         <f t="shared" ca="1" si="4"/>
-        <v>193.24449630775439</v>
-      </c>
-      <c r="K27" s="314">
+        <v>189.25415926230835</v>
+      </c>
+      <c r="K27" s="313">
         <f t="shared" ca="1" si="5"/>
-        <v>4274.9613619169686</v>
-      </c>
-      <c r="L27" s="314"/>
+        <v>4186.5154739201571</v>
+      </c>
+      <c r="L27" s="313"/>
       <c r="M27" s="77"/>
       <c r="N27" s="24"/>
       <c r="O27" s="226">
         <v>2</v>
       </c>
-      <c r="P27" s="324"/>
+      <c r="P27" s="323"/>
       <c r="Q27" s="24"/>
       <c r="R27" s="24"/>
       <c r="S27" s="24"/>
@@ -24238,19 +24234,19 @@
       </c>
       <c r="J28" s="307">
         <f t="shared" ref="J28:J36" ca="1" si="11">IF(C28="","",I27+J27)</f>
-        <v>218.87320516334364</v>
-      </c>
-      <c r="K28" s="314">
+        <v>214.35709633677948</v>
+      </c>
+      <c r="K28" s="313">
         <f t="shared" ref="K28:K36" ca="1" si="12">IF(C28="","",J28 * D28+K27)</f>
-        <v>6792.0032212954211</v>
-      </c>
-      <c r="L28" s="314"/>
+        <v>6651.6220817931207</v>
+      </c>
+      <c r="L28" s="313"/>
       <c r="M28" s="77"/>
       <c r="N28" s="24"/>
       <c r="O28" s="226">
         <v>3</v>
       </c>
-      <c r="P28" s="324"/>
+      <c r="P28" s="323"/>
       <c r="Q28" s="24"/>
       <c r="R28" s="24"/>
       <c r="S28" s="24"/>
@@ -24291,17 +24287,17 @@
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="K29" s="314" t="str">
+      <c r="K29" s="313" t="str">
         <f t="shared" si="12"/>
         <v/>
       </c>
-      <c r="L29" s="314"/>
+      <c r="L29" s="313"/>
       <c r="M29" s="77"/>
       <c r="N29" s="24"/>
       <c r="O29" s="226">
         <v>4</v>
       </c>
-      <c r="P29" s="324"/>
+      <c r="P29" s="323"/>
       <c r="Q29" s="24"/>
       <c r="R29" s="24"/>
       <c r="S29" s="24"/>
@@ -24342,17 +24338,17 @@
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="K30" s="314" t="str">
+      <c r="K30" s="313" t="str">
         <f t="shared" si="12"/>
         <v/>
       </c>
-      <c r="L30" s="314"/>
+      <c r="L30" s="313"/>
       <c r="M30" s="77"/>
       <c r="N30" s="24"/>
       <c r="O30" s="226">
         <v>5</v>
       </c>
-      <c r="P30" s="324"/>
+      <c r="P30" s="323"/>
       <c r="Q30" s="24"/>
       <c r="R30" s="24"/>
       <c r="S30" s="24"/>
@@ -24393,17 +24389,17 @@
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="K31" s="314" t="str">
+      <c r="K31" s="313" t="str">
         <f t="shared" si="12"/>
         <v/>
       </c>
-      <c r="L31" s="314"/>
+      <c r="L31" s="313"/>
       <c r="M31" s="77"/>
       <c r="N31" s="24"/>
       <c r="O31" s="226">
         <v>6</v>
       </c>
-      <c r="P31" s="324"/>
+      <c r="P31" s="323"/>
       <c r="Q31" s="24"/>
       <c r="R31" s="24"/>
       <c r="S31" s="24"/>
@@ -24444,17 +24440,17 @@
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="K32" s="314" t="str">
+      <c r="K32" s="313" t="str">
         <f t="shared" si="12"/>
         <v/>
       </c>
-      <c r="L32" s="314"/>
+      <c r="L32" s="313"/>
       <c r="M32" s="77"/>
       <c r="N32" s="24"/>
       <c r="O32" s="226">
         <v>7</v>
       </c>
-      <c r="P32" s="324"/>
+      <c r="P32" s="323"/>
       <c r="Q32" s="24"/>
       <c r="R32" s="24"/>
       <c r="S32" s="24"/>
@@ -24495,17 +24491,17 @@
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="K33" s="314" t="str">
+      <c r="K33" s="313" t="str">
         <f t="shared" si="12"/>
         <v/>
       </c>
-      <c r="L33" s="314"/>
+      <c r="L33" s="313"/>
       <c r="M33" s="77"/>
       <c r="N33" s="24"/>
       <c r="O33" s="226">
         <v>8</v>
       </c>
-      <c r="P33" s="324"/>
+      <c r="P33" s="323"/>
       <c r="Q33" s="24"/>
       <c r="R33" s="24"/>
       <c r="S33" s="24"/>
@@ -24546,17 +24542,17 @@
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="K34" s="314" t="str">
+      <c r="K34" s="313" t="str">
         <f t="shared" si="12"/>
         <v/>
       </c>
-      <c r="L34" s="314"/>
+      <c r="L34" s="313"/>
       <c r="M34" s="77"/>
       <c r="N34" s="24"/>
       <c r="O34" s="226">
         <v>9</v>
       </c>
-      <c r="P34" s="324"/>
+      <c r="P34" s="323"/>
       <c r="Q34" s="24"/>
       <c r="R34" s="24"/>
       <c r="S34" s="24"/>
@@ -24597,17 +24593,17 @@
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="K35" s="314" t="str">
+      <c r="K35" s="313" t="str">
         <f t="shared" si="12"/>
         <v/>
       </c>
-      <c r="L35" s="314"/>
+      <c r="L35" s="313"/>
       <c r="M35" s="77"/>
       <c r="N35" s="24"/>
       <c r="O35" s="226">
         <v>10</v>
       </c>
-      <c r="P35" s="324"/>
+      <c r="P35" s="323"/>
       <c r="Q35" s="24"/>
       <c r="R35" s="24"/>
       <c r="S35" s="24"/>
@@ -24648,17 +24644,17 @@
         <f t="shared" si="11"/>
         <v/>
       </c>
-      <c r="K36" s="315" t="str">
+      <c r="K36" s="314" t="str">
         <f t="shared" si="12"/>
         <v/>
       </c>
-      <c r="L36" s="315"/>
+      <c r="L36" s="314"/>
       <c r="M36" s="77"/>
       <c r="N36" s="24"/>
       <c r="O36" s="227">
         <v>11</v>
       </c>
-      <c r="P36" s="325"/>
+      <c r="P36" s="324"/>
       <c r="Q36" s="24"/>
       <c r="R36" s="24"/>
       <c r="S36" s="24"/>
@@ -24701,18 +24697,18 @@
     <row r="38" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="35"/>
       <c r="B38" s="232"/>
-      <c r="C38" s="327" t="s">
+      <c r="C38" s="326" t="s">
         <v>195</v>
       </c>
-      <c r="D38" s="327"/>
-      <c r="E38" s="327"/>
-      <c r="F38" s="327"/>
-      <c r="G38" s="327"/>
-      <c r="H38" s="327"/>
-      <c r="I38" s="327"/>
-      <c r="J38" s="327"/>
-      <c r="K38" s="327"/>
-      <c r="L38" s="327"/>
+      <c r="D38" s="326"/>
+      <c r="E38" s="326"/>
+      <c r="F38" s="326"/>
+      <c r="G38" s="326"/>
+      <c r="H38" s="326"/>
+      <c r="I38" s="326"/>
+      <c r="J38" s="326"/>
+      <c r="K38" s="326"/>
+      <c r="L38" s="326"/>
       <c r="M38" s="77"/>
       <c r="N38" s="24"/>
       <c r="O38" s="191" t="s">
@@ -24764,17 +24760,17 @@
       <c r="A40" s="35"/>
       <c r="B40" s="232"/>
       <c r="C40" s="272"/>
-      <c r="D40" s="328" t="s">
+      <c r="D40" s="327" t="s">
         <v>174</v>
       </c>
-      <c r="E40" s="329"/>
+      <c r="E40" s="328"/>
       <c r="F40" s="272"/>
       <c r="G40" s="272"/>
       <c r="H40" s="272"/>
-      <c r="I40" s="328" t="s">
+      <c r="I40" s="327" t="s">
         <v>174</v>
       </c>
-      <c r="J40" s="329"/>
+      <c r="J40" s="328"/>
       <c r="K40" s="272"/>
       <c r="L40" s="272"/>
       <c r="M40" s="287"/>
@@ -24798,19 +24794,19 @@
       <c r="A41" s="35"/>
       <c r="B41" s="232"/>
       <c r="C41" s="273"/>
-      <c r="D41" s="330" t="s">
+      <c r="D41" s="329" t="s">
         <v>200</v>
       </c>
-      <c r="E41" s="330"/>
+      <c r="E41" s="329"/>
       <c r="F41" s="273" t="s">
         <v>196</v>
       </c>
       <c r="G41" s="273"/>
       <c r="H41" s="244"/>
-      <c r="I41" s="330" t="s">
+      <c r="I41" s="329" t="s">
         <v>201</v>
       </c>
-      <c r="J41" s="330"/>
+      <c r="J41" s="329"/>
       <c r="K41" s="244" t="s">
         <v>196</v>
       </c>
@@ -24893,7 +24889,7 @@
       </c>
       <c r="F43" s="278">
         <f>IF(ISNUMBER(F24),F24,"")</f>
-        <v>430.46499999999997</v>
+        <v>421.49</v>
       </c>
       <c r="G43" s="279" t="e">
         <f>IF(ISNUMBER(F43),E43/F43-1,"")</f>
@@ -24904,7 +24900,7 @@
       <c r="J43" s="276"/>
       <c r="K43" s="278">
         <f ca="1">I24</f>
-        <v>72.824218936006218</v>
+        <v>71.308726197326649</v>
       </c>
       <c r="L43" s="279">
         <f t="shared" ref="L43" ca="1" si="13">IF(ISNUMBER(K43),I43/K43-1,"")</f>
@@ -24916,7 +24912,7 @@
       </c>
       <c r="N43" s="24"/>
       <c r="O43" s="225"/>
-      <c r="P43" s="323" t="s">
+      <c r="P43" s="322" t="s">
         <v>213</v>
       </c>
       <c r="Q43" s="24"/>
@@ -24944,7 +24940,7 @@
       </c>
       <c r="F44" s="278">
         <f t="shared" ref="F44:F55" si="15">IF(ISNUMBER(F25),F25,"")</f>
-        <v>554.33450000000005</v>
+        <v>542.91700000000003</v>
       </c>
       <c r="G44" s="279" t="e">
         <f t="shared" ref="G44:G55" si="16">IF(ISNUMBER(F44),E44/F44-1,"")</f>
@@ -24955,7 +24951,7 @@
       <c r="J44" s="281"/>
       <c r="K44" s="278">
         <f t="shared" ref="K44:K55" ca="1" si="17">I25</f>
-        <v>71.714063094992355</v>
+        <v>70.239801392449749</v>
       </c>
       <c r="L44" s="279">
         <f t="shared" ref="L44:L55" ca="1" si="18">IF(ISNUMBER(K44),I44/K44-1,"")</f>
@@ -24969,7 +24965,7 @@
       <c r="O44" s="226" t="s">
         <v>186</v>
       </c>
-      <c r="P44" s="324"/>
+      <c r="P44" s="323"/>
       <c r="Q44" s="24"/>
       <c r="R44" s="24"/>
       <c r="S44" s="24"/>
@@ -24995,7 +24991,7 @@
       </c>
       <c r="F45" s="278">
         <f t="shared" si="15"/>
-        <v>556.17650000000003</v>
+        <v>544.72900000000004</v>
       </c>
       <c r="G45" s="279" t="e">
         <f t="shared" si="16"/>
@@ -25006,7 +25002,7 @@
       <c r="J45" s="281"/>
       <c r="K45" s="278">
         <f t="shared" ca="1" si="17"/>
-        <v>48.706214276755809</v>
+        <v>47.705631672531936</v>
       </c>
       <c r="L45" s="279">
         <f t="shared" ca="1" si="18"/>
@@ -25020,7 +25016,7 @@
       <c r="O45" s="226">
         <v>1</v>
       </c>
-      <c r="P45" s="324"/>
+      <c r="P45" s="323"/>
       <c r="Q45" s="24"/>
       <c r="R45" s="24"/>
       <c r="S45" s="24"/>
@@ -25046,7 +25042,7 @@
       </c>
       <c r="F46" s="278">
         <f t="shared" si="15"/>
-        <v>559.8605</v>
+        <v>548.35299999999995</v>
       </c>
       <c r="G46" s="279" t="e">
         <f t="shared" si="16"/>
@@ -25057,7 +25053,7 @@
       <c r="J46" s="281"/>
       <c r="K46" s="278">
         <f t="shared" ca="1" si="17"/>
-        <v>25.628708855589242</v>
+        <v>25.102937074471132</v>
       </c>
       <c r="L46" s="279">
         <f t="shared" ca="1" si="18"/>
@@ -25071,7 +25067,7 @@
       <c r="O46" s="226">
         <v>2</v>
       </c>
-      <c r="P46" s="324"/>
+      <c r="P46" s="323"/>
       <c r="Q46" s="24"/>
       <c r="R46" s="24"/>
       <c r="S46" s="24"/>
@@ -25122,7 +25118,7 @@
       <c r="O47" s="226">
         <v>3</v>
       </c>
-      <c r="P47" s="324"/>
+      <c r="P47" s="323"/>
       <c r="Q47" s="24"/>
       <c r="R47" s="24"/>
       <c r="S47" s="24"/>
@@ -25173,7 +25169,7 @@
       <c r="O48" s="226">
         <v>4</v>
       </c>
-      <c r="P48" s="324"/>
+      <c r="P48" s="323"/>
       <c r="Q48" s="24"/>
       <c r="R48" s="24"/>
       <c r="S48" s="24"/>
@@ -25224,7 +25220,7 @@
       <c r="O49" s="226">
         <v>5</v>
       </c>
-      <c r="P49" s="324"/>
+      <c r="P49" s="323"/>
       <c r="Q49" s="24"/>
       <c r="R49" s="24"/>
       <c r="S49" s="24"/>
@@ -25275,7 +25271,7 @@
       <c r="O50" s="226">
         <v>6</v>
       </c>
-      <c r="P50" s="324"/>
+      <c r="P50" s="323"/>
       <c r="Q50" s="24"/>
       <c r="R50" s="24"/>
       <c r="S50" s="24"/>
@@ -25326,7 +25322,7 @@
       <c r="O51" s="226">
         <v>7</v>
       </c>
-      <c r="P51" s="324"/>
+      <c r="P51" s="323"/>
       <c r="Q51" s="24"/>
       <c r="R51" s="24"/>
       <c r="S51" s="24"/>
@@ -25377,7 +25373,7 @@
       <c r="O52" s="226">
         <v>8</v>
       </c>
-      <c r="P52" s="324"/>
+      <c r="P52" s="323"/>
       <c r="Q52" s="24"/>
       <c r="R52" s="24"/>
       <c r="S52" s="24"/>
@@ -25428,7 +25424,7 @@
       <c r="O53" s="226">
         <v>9</v>
       </c>
-      <c r="P53" s="324"/>
+      <c r="P53" s="323"/>
       <c r="Q53" s="24"/>
       <c r="R53" s="24"/>
       <c r="S53" s="24"/>
@@ -25479,7 +25475,7 @@
       <c r="O54" s="226">
         <v>10</v>
       </c>
-      <c r="P54" s="324"/>
+      <c r="P54" s="323"/>
       <c r="Q54" s="24"/>
       <c r="R54" s="24"/>
       <c r="S54" s="24"/>
@@ -25530,7 +25526,7 @@
       <c r="O55" s="227">
         <v>11</v>
       </c>
-      <c r="P55" s="325"/>
+      <c r="P55" s="324"/>
       <c r="Q55" s="24"/>
       <c r="R55" s="24"/>
       <c r="S55" s="24"/>
@@ -25573,21 +25569,21 @@
     <row r="57" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="253"/>
       <c r="B57" s="232"/>
-      <c r="C57" s="311" t="s">
+      <c r="C57" s="310" t="s">
         <v>209</v>
       </c>
-      <c r="D57" s="311"/>
-      <c r="E57" s="311"/>
+      <c r="D57" s="310"/>
+      <c r="E57" s="310"/>
       <c r="F57" s="181" t="s">
         <v>207</v>
       </c>
       <c r="G57" s="231" t="s">
         <v>208</v>
       </c>
-      <c r="H57" s="312" t="s">
+      <c r="H57" s="311" t="s">
         <v>210</v>
       </c>
-      <c r="I57" s="312"/>
+      <c r="I57" s="311"/>
       <c r="J57" s="244" t="s">
         <v>204</v>
       </c>
@@ -25618,11 +25614,11 @@
       <c r="E58" s="232"/>
       <c r="F58" s="255"/>
       <c r="G58" s="256"/>
-      <c r="H58" s="313">
+      <c r="H58" s="312">
         <f ca="1">I12</f>
-        <v>218.87320516334364</v>
-      </c>
-      <c r="I58" s="313"/>
+        <v>214.35709633677951</v>
+      </c>
+      <c r="I58" s="312"/>
       <c r="J58" s="299">
         <f ca="1">F58/H58-1</f>
         <v>-1</v>
@@ -27330,14 +27326,14 @@
       <c r="C1" s="197" t="s">
         <v>131</v>
       </c>
-      <c r="D1" s="331" t="str">
+      <c r="D1" s="330" t="str">
         <f>+IF('Site Ground Motions'!E1="","",'Site Ground Motions'!E1)</f>
         <v/>
       </c>
-      <c r="E1" s="332"/>
-      <c r="F1" s="332"/>
-      <c r="G1" s="332"/>
-      <c r="H1" s="333"/>
+      <c r="E1" s="331"/>
+      <c r="F1" s="331"/>
+      <c r="G1" s="331"/>
+      <c r="H1" s="332"/>
       <c r="I1" s="219" t="s">
         <v>132</v>
       </c>
@@ -27375,14 +27371,14 @@
       <c r="C2" s="197" t="s">
         <v>135</v>
       </c>
-      <c r="D2" s="331" t="str">
+      <c r="D2" s="330" t="str">
         <f>+IF('Site Ground Motions'!E2="","",'Site Ground Motions'!E2)</f>
         <v/>
       </c>
-      <c r="E2" s="332"/>
-      <c r="F2" s="332"/>
-      <c r="G2" s="332"/>
-      <c r="H2" s="333"/>
+      <c r="E2" s="331"/>
+      <c r="F2" s="331"/>
+      <c r="G2" s="331"/>
+      <c r="H2" s="332"/>
       <c r="I2" s="219" t="s">
         <v>136</v>
       </c>
@@ -27420,14 +27416,14 @@
       <c r="C3" s="197" t="s">
         <v>138</v>
       </c>
-      <c r="D3" s="331" t="str">
+      <c r="D3" s="330" t="str">
         <f>+IF('Site Ground Motions'!E3="","",'Site Ground Motions'!E3)</f>
         <v/>
       </c>
-      <c r="E3" s="332"/>
-      <c r="F3" s="332"/>
-      <c r="G3" s="332"/>
-      <c r="H3" s="333"/>
+      <c r="E3" s="331"/>
+      <c r="F3" s="331"/>
+      <c r="G3" s="331"/>
+      <c r="H3" s="332"/>
       <c r="I3" s="219" t="s">
         <v>139</v>
       </c>
@@ -27456,13 +27452,13 @@
       <c r="C4" s="197" t="s">
         <v>141</v>
       </c>
-      <c r="D4" s="331" t="s">
+      <c r="D4" s="330" t="s">
         <v>159</v>
       </c>
-      <c r="E4" s="332"/>
-      <c r="F4" s="332"/>
-      <c r="G4" s="332"/>
-      <c r="H4" s="333"/>
+      <c r="E4" s="331"/>
+      <c r="F4" s="331"/>
+      <c r="G4" s="331"/>
+      <c r="H4" s="332"/>
       <c r="I4" s="219" t="s">
         <v>136</v>
       </c>
@@ -27505,10 +27501,10 @@
       <c r="A6" s="7"/>
       <c r="K6" s="8"/>
       <c r="L6" s="24"/>
-      <c r="M6" s="339" t="s">
+      <c r="M6" s="338" t="s">
         <v>164</v>
       </c>
-      <c r="N6" s="339"/>
+      <c r="N6" s="338"/>
       <c r="O6" s="24"/>
       <c r="P6" s="24"/>
       <c r="Q6" s="24"/>
@@ -27580,7 +27576,7 @@
       </c>
       <c r="D9" s="178">
         <f>+'Vertical Distribution'!E9</f>
-        <v>2100.8365000000003</v>
+        <v>2057.489</v>
       </c>
       <c r="E9" s="232"/>
       <c r="F9" s="238"/>
@@ -27616,7 +27612,7 @@
       </c>
       <c r="G10" s="178">
         <f ca="1">+'Vertical Distribution'!I12</f>
-        <v>218.87320516334364</v>
+        <v>214.35709633677951</v>
       </c>
       <c r="H10" s="10"/>
       <c r="I10" s="10"/>
@@ -27744,12 +27740,12 @@
       <c r="A15" s="97"/>
       <c r="B15" s="181">
         <f>SUM(B18:B28)</f>
-        <v>2100.8365000000003</v>
+        <v>2057.489</v>
       </c>
       <c r="C15" s="232"/>
       <c r="D15" s="181">
         <f ca="1">SUM(D18:D28)</f>
-        <v>218.87320516334364</v>
+        <v>214.35709633677948</v>
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
@@ -27861,46 +27857,46 @@
       </c>
       <c r="B18" s="296">
         <f>IF(A18="Ground","—",IF(A18="","",'Vertical Distribution'!F24))</f>
-        <v>430.46499999999997</v>
+        <v>421.49</v>
       </c>
       <c r="C18" s="185">
         <f>B18</f>
-        <v>430.46499999999997</v>
+        <v>421.49</v>
       </c>
       <c r="D18" s="185">
         <f ca="1">+'Vertical Distribution'!I24</f>
-        <v>72.824218936006218</v>
+        <v>71.308726197326649</v>
       </c>
       <c r="E18" s="185">
         <f ca="1">D18</f>
-        <v>72.824218936006218</v>
+        <v>71.308726197326649</v>
       </c>
       <c r="F18" s="230">
         <f ca="1">E18 / C18</f>
-        <v>0.16917570287016651</v>
+        <v>0.16918248641089148</v>
       </c>
       <c r="G18" s="185">
         <f ca="1">F18 * B18</f>
-        <v>72.824218936006218</v>
+        <v>71.308726197326649</v>
       </c>
       <c r="H18" s="185">
         <f ca="1">0.2 * $C$12 * $F$12 * B18</f>
-        <v>58.301743395466666</v>
+        <v>57.086178490133342</v>
       </c>
       <c r="I18" s="185">
         <f ca="1">0.4 * $C$12 * $F$12 * B18</f>
-        <v>116.60348679093333</v>
+        <v>114.17235698026668</v>
       </c>
       <c r="J18" s="186">
         <f ca="1">IF(I18 &lt; MAX(G18, H18), I18, MAX(G18, H18))</f>
-        <v>72.824218936006218</v>
+        <v>71.308726197326649</v>
       </c>
       <c r="K18" s="297">
         <f ca="1">J18/B18</f>
-        <v>0.16917570287016651</v>
+        <v>0.16918248641089148</v>
       </c>
       <c r="L18" s="37"/>
-      <c r="M18" s="363" t="s">
+      <c r="M18" s="362" t="s">
         <v>212</v>
       </c>
       <c r="N18" s="24"/>
@@ -27920,46 +27916,46 @@
       </c>
       <c r="B19" s="185">
         <f>IF(A19="Ground","—",IF(A19="","",'Vertical Distribution'!F25))</f>
-        <v>554.33450000000005</v>
+        <v>542.91700000000003</v>
       </c>
       <c r="C19" s="181">
         <f>IF(A19="Ground","—",IF(A19="","",C18 + B19))</f>
-        <v>984.79950000000008</v>
+        <v>964.40700000000004</v>
       </c>
       <c r="D19" s="185">
         <f ca="1">IF(A19="Ground","—",IF(A19="","",'Vertical Distribution'!I25))</f>
-        <v>71.714063094992355</v>
+        <v>70.239801392449749</v>
       </c>
       <c r="E19" s="181">
         <f ca="1">IF(A19="Ground","—",IF(A19="","",E18 + D19))</f>
-        <v>144.53828203099857</v>
+        <v>141.5485275897764</v>
       </c>
       <c r="F19" s="230">
         <f ca="1">IF(A19="Ground","—",IF(A19="","",E19/C19))</f>
-        <v>0.14676924798499447</v>
+        <v>0.14677260491657193</v>
       </c>
       <c r="G19" s="185">
         <f ca="1">IF(A19="Ground","—",IF(A19="","",F19*B19))</f>
-        <v>81.35925769713792</v>
+        <v>79.68534234349049</v>
       </c>
       <c r="H19" s="185">
         <f ca="1">IF(A19="Ground","—",IF(A19="","",0.2*$C$12*$F$12*B19))</f>
-        <v>75.078502954373349</v>
+        <v>73.532128324106679</v>
       </c>
       <c r="I19" s="185">
         <f ca="1">IF(A19="Ground","—",IF(A19="","",0.4*$C$12*$F$12*B19))</f>
-        <v>150.1570059087467</v>
+        <v>147.06425664821336</v>
       </c>
       <c r="J19" s="186">
         <f ca="1">IF(A19="Ground","—",IF(A19="","",IF(I19&lt;MAX(G19,H19),I19,MAX(G19,H19))))</f>
-        <v>81.35925769713792</v>
+        <v>79.68534234349049</v>
       </c>
       <c r="K19" s="297">
         <f ca="1">IF(A19="Ground","—",IF(A19="","",J19/B19))</f>
-        <v>0.14676924798499447</v>
+        <v>0.14677260491657193</v>
       </c>
       <c r="L19" s="24"/>
-      <c r="M19" s="363"/>
+      <c r="M19" s="362"/>
       <c r="N19" s="24"/>
       <c r="O19" s="24"/>
       <c r="P19" s="24"/>
@@ -27977,46 +27973,46 @@
       </c>
       <c r="B20" s="185">
         <f>IF(A20="Ground","—",IF(A20="","",'Vertical Distribution'!F26))</f>
-        <v>556.17650000000003</v>
+        <v>544.72900000000004</v>
       </c>
       <c r="C20" s="181">
         <f t="shared" ref="C20:C30" si="0">IF(A20="Ground","—",IF(A20="","",C19 + B20))</f>
-        <v>1540.9760000000001</v>
+        <v>1509.136</v>
       </c>
       <c r="D20" s="185">
         <f ca="1">IF(A20="Ground","—",IF(A20="","",'Vertical Distribution'!I26))</f>
-        <v>48.706214276755809</v>
+        <v>47.705631672531936</v>
       </c>
       <c r="E20" s="181">
         <f t="shared" ref="E20:E30" ca="1" si="1">IF(A20="Ground","—",IF(A20="","",E19 + D20))</f>
-        <v>193.24449630775439</v>
+        <v>189.25415926230835</v>
       </c>
       <c r="F20" s="230">
         <f t="shared" ref="F20:F30" ca="1" si="2">IF(A20="Ground","—",IF(A20="","",E20/C20))</f>
-        <v>0.12540396236395271</v>
+        <v>0.12540563558374351</v>
       </c>
       <c r="G20" s="185">
         <f t="shared" ref="G20:G30" ca="1" si="3">IF(A20="Ground","—",IF(A20="","",F20*B20))</f>
-        <v>69.746736873714951</v>
+        <v>68.312086465897025</v>
       </c>
       <c r="H20" s="185">
         <f t="shared" ref="H20:H30" ca="1" si="4">IF(A20="Ground","—",IF(A20="","",0.2*$C$12*$F$12*B20))</f>
-        <v>75.327981567813339</v>
+        <v>73.777543767946682</v>
       </c>
       <c r="I20" s="185">
         <f t="shared" ref="I20:I30" ca="1" si="5">IF(A20="Ground","—",IF(A20="","",0.4*$C$12*$F$12*B20))</f>
-        <v>150.65596313562668</v>
+        <v>147.55508753589336</v>
       </c>
       <c r="J20" s="186">
         <f t="shared" ref="J20:J30" ca="1" si="6">IF(A20="Ground","—",IF(A20="","",IF(I20&lt;MAX(G20,H20),I20,MAX(G20,H20))))</f>
-        <v>75.327981567813339</v>
+        <v>73.777543767946682</v>
       </c>
       <c r="K20" s="297">
         <f t="shared" ref="K20:K30" ca="1" si="7">IF(A20="Ground","—",IF(A20="","",J20/B20))</f>
         <v>0.13543898666666668</v>
       </c>
       <c r="L20" s="24"/>
-      <c r="M20" s="363"/>
+      <c r="M20" s="362"/>
       <c r="N20" s="24"/>
       <c r="O20" s="24"/>
       <c r="P20" s="24"/>
@@ -28034,46 +28030,46 @@
       </c>
       <c r="B21" s="185">
         <f>IF(A21="Ground","—",IF(A21="","",'Vertical Distribution'!F27))</f>
-        <v>559.8605</v>
+        <v>548.35299999999995</v>
       </c>
       <c r="C21" s="181">
         <f t="shared" si="0"/>
-        <v>2100.8365000000003</v>
+        <v>2057.489</v>
       </c>
       <c r="D21" s="185">
         <f ca="1">IF(A21="Ground","—",IF(A21="","",'Vertical Distribution'!I27))</f>
-        <v>25.628708855589242</v>
+        <v>25.102937074471132</v>
       </c>
       <c r="E21" s="181">
         <f t="shared" ca="1" si="1"/>
-        <v>218.87320516334364</v>
+        <v>214.35709633677948</v>
       </c>
       <c r="F21" s="230">
         <f t="shared" ca="1" si="2"/>
-        <v>0.10418383589743591</v>
+        <v>0.10418383589743589</v>
       </c>
       <c r="G21" s="185">
         <f t="shared" ca="1" si="3"/>
-        <v>58.328414457456418</v>
+        <v>57.129518965866659</v>
       </c>
       <c r="H21" s="185">
         <f t="shared" ca="1" si="4"/>
-        <v>75.826938794693334</v>
+        <v>74.268374655626673</v>
       </c>
       <c r="I21" s="185">
         <f t="shared" ca="1" si="5"/>
-        <v>151.65387758938667</v>
+        <v>148.53674931125335</v>
       </c>
       <c r="J21" s="186">
         <f t="shared" ca="1" si="6"/>
-        <v>75.826938794693334</v>
+        <v>74.268374655626673</v>
       </c>
       <c r="K21" s="297">
         <f t="shared" ca="1" si="7"/>
         <v>0.13543898666666668</v>
       </c>
       <c r="L21" s="24"/>
-      <c r="M21" s="363"/>
+      <c r="M21" s="362"/>
       <c r="N21" s="24"/>
       <c r="O21" s="24"/>
       <c r="P21" s="24"/>
@@ -28130,7 +28126,7 @@
         <v>—</v>
       </c>
       <c r="L22" s="24"/>
-      <c r="M22" s="363"/>
+      <c r="M22" s="362"/>
       <c r="N22" s="24"/>
       <c r="O22" s="24"/>
       <c r="P22" s="24"/>
@@ -28187,7 +28183,7 @@
         <v/>
       </c>
       <c r="L23" s="24"/>
-      <c r="M23" s="363"/>
+      <c r="M23" s="362"/>
       <c r="N23" s="24"/>
       <c r="O23" s="24"/>
       <c r="P23" s="24"/>
@@ -28244,7 +28240,7 @@
         <v/>
       </c>
       <c r="L24" s="24"/>
-      <c r="M24" s="363"/>
+      <c r="M24" s="362"/>
       <c r="N24" s="24"/>
       <c r="O24" s="24"/>
       <c r="P24" s="24"/>
@@ -28301,7 +28297,7 @@
         <v/>
       </c>
       <c r="L25" s="24"/>
-      <c r="M25" s="363"/>
+      <c r="M25" s="362"/>
       <c r="N25" s="24"/>
       <c r="O25" s="24"/>
       <c r="P25" s="24"/>
@@ -28358,7 +28354,7 @@
         <v/>
       </c>
       <c r="L26" s="24"/>
-      <c r="M26" s="363"/>
+      <c r="M26" s="362"/>
       <c r="N26" s="24"/>
       <c r="O26" s="24"/>
       <c r="P26" s="24"/>
@@ -28415,7 +28411,7 @@
         <v/>
       </c>
       <c r="L27" s="24"/>
-      <c r="M27" s="363"/>
+      <c r="M27" s="362"/>
       <c r="N27" s="24"/>
       <c r="O27" s="24"/>
       <c r="P27" s="24"/>
@@ -28472,7 +28468,7 @@
         <v/>
       </c>
       <c r="L28" s="24"/>
-      <c r="M28" s="363"/>
+      <c r="M28" s="362"/>
       <c r="N28" s="24"/>
       <c r="O28" s="24"/>
       <c r="P28" s="24"/>
@@ -28529,7 +28525,7 @@
         <v/>
       </c>
       <c r="L29" s="24"/>
-      <c r="M29" s="363"/>
+      <c r="M29" s="362"/>
       <c r="N29" s="24"/>
       <c r="O29" s="24"/>
       <c r="P29" s="24"/>
@@ -28586,7 +28582,7 @@
         <v/>
       </c>
       <c r="L30" s="24"/>
-      <c r="M30" s="363"/>
+      <c r="M30" s="362"/>
       <c r="N30" s="24"/>
       <c r="O30" s="24"/>
       <c r="P30" s="24"/>

</xml_diff>